<commit_message>
Publish the Streamlit UI, exploratory analysis, and PySD v3 live-simulation stack.
</commit_message>
<xml_diff>
--- a/Input and Output Streamlit.xlsx
+++ b/Input and Output Streamlit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://supsi-my.sharepoint.com/personal/matteo_palucci_supsi_ch/Documents/Desktop/SEneCa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="8_{19367E20-36FD-4AD5-B7E8-1C9AFB5E8597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57C5C7E3-3EE3-408E-B989-F3A5E641CFC3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{66AB5E74-7B18-4269-B928-99CA671C10DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{B9177ACD-C732-4210-952B-EADD8A8D5047}"/>
+    <workbookView xWindow="13740" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="705" activeTab="5" xr2:uid="{B9177ACD-C732-4210-952B-EADD8A8D5047}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Output Risc e Risanamento" sheetId="3" r:id="rId3"/>
     <sheet name="Output Veicoli" sheetId="4" r:id="rId4"/>
     <sheet name="Output Elettricità" sheetId="5" r:id="rId5"/>
+    <sheet name="Exploratory analysis" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="233">
   <si>
     <t>Max</t>
   </si>
@@ -674,6 +675,93 @@
   </si>
   <si>
     <t>Costo annuale upgrade rete bassa tensione</t>
+  </si>
+  <si>
+    <t>Policy</t>
+  </si>
+  <si>
+    <t>PV uncertain cost</t>
+  </si>
+  <si>
+    <t>PV uncertain remuneration</t>
+  </si>
+  <si>
+    <t>Retrofit uncertain cost</t>
+  </si>
+  <si>
+    <t>Interest rate uncertainty</t>
+  </si>
+  <si>
+    <t>Import price uncertainty</t>
+  </si>
+  <si>
+    <t>Battery uncertain cost</t>
+  </si>
+  <si>
+    <t>Construction rate uncertainty</t>
+  </si>
+  <si>
+    <t>Demolition rate uncertainty</t>
+  </si>
+  <si>
+    <t>Industry demand uncertainty</t>
+  </si>
+  <si>
+    <t>Tertiary demand uncertainty</t>
+  </si>
+  <si>
+    <t>Oil/gas lifetime uncertainty</t>
+  </si>
+  <si>
+    <t>Wood/pellet lifetime uncertainty</t>
+  </si>
+  <si>
+    <t>HP lifetime uncertainty</t>
+  </si>
+  <si>
+    <t>Oil/gas carrier cost uncertainty</t>
+  </si>
+  <si>
+    <t>Wood/pellet carrier cost uncertainty</t>
+  </si>
+  <si>
+    <t>HP cost uncertainty</t>
+  </si>
+  <si>
+    <t>HP efficiency uncertainty</t>
+  </si>
+  <si>
+    <t>Uncertainty</t>
+  </si>
+  <si>
+    <t>Cantonal PV support</t>
+  </si>
+  <si>
+    <t>Renewable heating incentives</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>Inequality index levy</t>
+  </si>
+  <si>
+    <t>Inequality index CO2 tax</t>
+  </si>
+  <si>
+    <t>Inequality index cost</t>
+  </si>
+  <si>
+    <t>Average cost</t>
+  </si>
+  <si>
+    <t>PV annual production</t>
+  </si>
+  <si>
+    <t>Average net specific consumption</t>
+  </si>
+  <si>
+    <t>Cumulative cantonal spending</t>
   </si>
 </sst>
 </file>
@@ -3038,6 +3126,397 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9233D4C2-B5A4-4D91-9DDD-8654D3E63A97}">
+  <dimension ref="A1:H39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="27.41796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.20703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="8.20703125" customWidth="1"/>
+    <col min="18" max="18" width="12.5234375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0.3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0.2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B5">
+        <v>50</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="G8">
+        <f>PRODUCT(E2:E8)</f>
+        <v>128</v>
+      </c>
+      <c r="H8">
+        <f>G8*H7</f>
+        <v>6400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="E10" s="2"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B13">
+        <v>-0.2</v>
+      </c>
+      <c r="C13">
+        <v>0.2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B14">
+        <v>-0.2</v>
+      </c>
+      <c r="C14">
+        <v>0.2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B15">
+        <v>-0.1</v>
+      </c>
+      <c r="C15">
+        <v>0.1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16">
+        <v>-0.3</v>
+      </c>
+      <c r="C16">
+        <v>0.3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17">
+        <v>-0.3</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18">
+        <v>-0.2</v>
+      </c>
+      <c r="C18">
+        <v>0.2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19">
+        <v>-0.2</v>
+      </c>
+      <c r="C19">
+        <v>0.2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20">
+        <v>-0.2</v>
+      </c>
+      <c r="C20">
+        <v>0.2</v>
+      </c>
+      <c r="D20" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21">
+        <v>-0.2</v>
+      </c>
+      <c r="C21">
+        <v>0.2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22">
+        <v>-0.2</v>
+      </c>
+      <c r="C22">
+        <v>0.2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23">
+        <v>-0.2</v>
+      </c>
+      <c r="C23">
+        <v>0.2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B24">
+        <v>-0.2</v>
+      </c>
+      <c r="C24">
+        <v>0.2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B25">
+        <v>-0.2</v>
+      </c>
+      <c r="C25">
+        <v>0.2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26">
+        <v>-0.2</v>
+      </c>
+      <c r="C26">
+        <v>0.2</v>
+      </c>
+      <c r="D26" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27">
+        <v>-0.2</v>
+      </c>
+      <c r="C27">
+        <v>0.2</v>
+      </c>
+      <c r="D27" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B28">
+        <v>-0.3</v>
+      </c>
+      <c r="C28">
+        <v>0.3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="B29">
+        <v>-0.2</v>
+      </c>
+      <c r="C29">
+        <v>0.2</v>
+      </c>
+      <c r="D29" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101002DA1C5DD1C76D544AACEF782C4501B75" ma:contentTypeVersion="19" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="e653d769d9bfe89dd5bdefbfba6c6e39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5c44f38a-956f-4897-8911-fab8683ac3ce" xmlns:ns3="3a2a3416-dcc9-40bd-acae-10337fdfc866" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="07aee1c0ca2ce908aaeda2f09eacdfad" ns2:_="" ns3:_="">

</xml_diff>

<commit_message>
Pysd v4, test scenario metadata
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Input and Output Streamlit.xlsx
+++ b/Input and Output Streamlit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://supsi-my.sharepoint.com/personal/matteo_palucci_supsi_ch/Documents/Desktop/SEneCa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66AB5E74-7B18-4269-B928-99CA671C10DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{66AB5E74-7B18-4269-B928-99CA671C10DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CC26676-4F75-495A-9B1A-F6081CADC53F}"/>
   <bookViews>
-    <workbookView xWindow="13740" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="705" activeTab="5" xr2:uid="{B9177ACD-C732-4210-952B-EADD8A8D5047}"/>
+    <workbookView xWindow="-110" yWindow="-21710" windowWidth="38620" windowHeight="21100" tabRatio="705" xr2:uid="{B9177ACD-C732-4210-952B-EADD8A8D5047}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="234">
   <si>
     <t>Max</t>
   </si>
@@ -762,6 +762,9 @@
   </si>
   <si>
     <t>Cumulative cantonal spending</t>
+  </si>
+  <si>
+    <t>Total PV electricity SC degree</t>
   </si>
 </sst>
 </file>
@@ -1143,7 +1146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C92CED1-ADF5-4E3A-8D95-AABCB30FA95C}">
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="13.47265625" bestFit="1" customWidth="1"/>
@@ -1264,42 +1267,38 @@
       <c r="K3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
       <c r="D4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I4" t="s">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="N4" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
         <v>1</v>
@@ -1308,27 +1307,27 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="G5">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="H5" t="s">
         <v>7</v>
       </c>
       <c r="I5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="J5">
         <v>3</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
@@ -1346,7 +1345,7 @@
         <v>7</v>
       </c>
       <c r="I6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J6">
         <v>3</v>
@@ -1357,7 +1356,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C7" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
@@ -1375,7 +1374,7 @@
         <v>7</v>
       </c>
       <c r="I7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J7">
         <v>3</v>
@@ -1386,25 +1385,25 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G8">
-        <v>50</v>
+        <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="J8">
         <v>3</v>
@@ -1415,145 +1414,145 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>4000</v>
+        <v>100</v>
       </c>
       <c r="G9">
-        <v>2000</v>
+        <v>50</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J9">
         <v>3</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>0.4</v>
+        <v>4000</v>
       </c>
       <c r="G10">
-        <v>0.2</v>
+        <v>2000</v>
       </c>
       <c r="H10" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="I10" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="J10">
         <v>3</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="N10" s="2" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>240</v>
+        <v>0.4</v>
       </c>
       <c r="G11">
-        <v>120</v>
+        <v>0.2</v>
       </c>
       <c r="H11" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="J11">
         <v>3</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M11" s="2"/>
+      <c r="N11" s="2" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>240</v>
+      </c>
+      <c r="G12">
+        <v>120</v>
+      </c>
+      <c r="H12" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
         <v>33</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>30</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>5</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" t="s">
         <v>49</v>
       </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
         <v>1</v>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-      <c r="H12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I12" t="s">
-        <v>57</v>
-      </c>
-      <c r="J12">
-        <v>2</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>2</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1562,162 +1561,177 @@
         <v>7</v>
       </c>
       <c r="I13" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J13">
-        <v>3</v>
-      </c>
-      <c r="L13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>158</v>
+        <v>62</v>
       </c>
       <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14">
         <v>1</v>
-      </c>
-      <c r="F14">
-        <v>4</v>
-      </c>
-      <c r="G14">
-        <v>2</v>
       </c>
       <c r="H14" t="s">
         <v>7</v>
       </c>
       <c r="I14" t="s">
-        <v>157</v>
+        <v>62</v>
       </c>
       <c r="J14">
-        <v>4</v>
-      </c>
-      <c r="M14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C15" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>158</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" t="s">
         <v>7</v>
       </c>
       <c r="I15" t="s">
+        <v>157</v>
+      </c>
+      <c r="J15">
+        <v>4</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" t="s">
         <v>56</v>
       </c>
-      <c r="J15">
+      <c r="J16">
         <v>2</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K16" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" t="s">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" t="s">
         <v>36</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>37</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>5</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D17" t="s">
         <v>68</v>
       </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
         <v>-5</v>
-      </c>
-      <c r="H16" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>5</v>
       </c>
       <c r="H17" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>5</v>
+      </c>
+      <c r="H18" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C19" t="s">
         <v>66</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>69</v>
       </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
         <v>0.03</v>
       </c>
-      <c r="G18">
+      <c r="G19">
         <v>0.01</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H19" t="s">
         <v>7</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I19" t="s">
         <v>70</v>
       </c>
-      <c r="J18">
+      <c r="J19">
         <v>4</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M19" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C19" t="s">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C20" t="s">
         <v>24</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D20" t="s">
         <v>6</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19">
-        <v>5</v>
-      </c>
-      <c r="H19" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="D20" t="s">
-        <v>9</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -1729,9 +1743,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="D21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1743,27 +1757,26 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C22" t="s">
-        <v>40</v>
-      </c>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="D22" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E22">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H22" t="s">
         <v>3</v>
       </c>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C23" t="s">
+        <v>40</v>
+      </c>
       <c r="D23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23">
         <v>-1</v>
@@ -1776,82 +1789,68 @@
       </c>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="D24" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24">
+        <v>-1</v>
+      </c>
+      <c r="F24">
+        <v>4</v>
+      </c>
+      <c r="H24" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="D25" t="s">
         <v>156</v>
       </c>
-      <c r="E24">
+      <c r="E25">
         <v>2</v>
       </c>
-      <c r="F24">
+      <c r="F25">
         <v>3</v>
       </c>
-      <c r="G24">
+      <c r="G25">
         <v>2</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H25" t="s">
         <v>63</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I25" t="s">
         <v>155</v>
       </c>
-      <c r="J24">
+      <c r="J25">
         <v>3</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M25" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="B25" t="s">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="B26" t="s">
         <v>41</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>12</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D26" t="s">
         <v>42</v>
       </c>
-      <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="B26" t="s">
+      <c r="M26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="B27" t="s">
         <v>43</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>44</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>183</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26" t="s">
-        <v>7</v>
-      </c>
-      <c r="I26" t="s">
-        <v>182</v>
-      </c>
-      <c r="J26">
-        <v>2</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="C27" t="s">
-        <v>184</v>
-      </c>
-      <c r="D27" t="s">
-        <v>185</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1866,7 +1865,7 @@
         <v>7</v>
       </c>
       <c r="I27" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="J27">
         <v>2</v>
@@ -1875,12 +1874,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C28" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D28" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1895,7 +1894,7 @@
         <v>7</v>
       </c>
       <c r="I28" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="J28">
         <v>2</v>
@@ -1904,12 +1903,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C29" t="s">
-        <v>44</v>
+        <v>187</v>
       </c>
       <c r="D29" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1924,7 +1923,7 @@
         <v>7</v>
       </c>
       <c r="I29" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J29">
         <v>2</v>
@@ -1933,12 +1932,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C30" t="s">
         <v>44</v>
       </c>
       <c r="D30" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -1953,19 +1952,21 @@
         <v>7</v>
       </c>
       <c r="I30" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J30">
         <v>2</v>
       </c>
-      <c r="N30" s="2"/>
-    </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="N30" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.55000000000000004">
       <c r="C31" t="s">
         <v>44</v>
       </c>
       <c r="D31" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1980,32 +1981,59 @@
         <v>7</v>
       </c>
       <c r="I31" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="J31">
         <v>2</v>
       </c>
       <c r="N31" s="2"/>
     </row>
-    <row r="33" spans="10:14" x14ac:dyDescent="0.55000000000000004">
-      <c r="J33" s="2" t="s">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>194</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>7</v>
+      </c>
+      <c r="I32" t="s">
+        <v>195</v>
+      </c>
+      <c r="J32">
+        <v>2</v>
+      </c>
+      <c r="N32" s="2"/>
+    </row>
+    <row r="34" spans="10:14" x14ac:dyDescent="0.55000000000000004">
+      <c r="J34" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K33" cm="1">
-        <f t="array" ref="K33">PRODUCT(IF(K2:K31=$J$33,$J$2:$J$31))</f>
+      <c r="K34" cm="1">
+        <f t="array" ref="K34">PRODUCT(IF(K2:K32=$J$34,$J$2:$J$32))</f>
         <v>324</v>
       </c>
-      <c r="L33" cm="1">
-        <f t="array" ref="L33">PRODUCT(IF(L2:L31=$J$33,$J$2:$J$31))</f>
+      <c r="L34" cm="1">
+        <f t="array" ref="L34">PRODUCT(IF(L2:L32=$J$34,$J$2:$J$32))</f>
         <v>729</v>
       </c>
-      <c r="M33" cm="1">
-        <f t="array" ref="M33">PRODUCT(IF(M2:M31=$J$33,$J$2:$J$31))</f>
+      <c r="M34" cm="1">
+        <f t="array" ref="M34">PRODUCT(IF(M2:M32=$J$34,$J$2:$J$32))</f>
         <v>144</v>
       </c>
-      <c r="N33" cm="1">
-        <f t="array" ref="N33">PRODUCT(IF(N2:N31=$J$33,$J$2:$J$31))</f>
-        <v>144</v>
+      <c r="N34" cm="1">
+        <f t="array" ref="N34">PRODUCT(IF(N2:N32=$J$34,$J$2:$J$32))</f>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -3128,7 +3156,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9233D4C2-B5A4-4D91-9DDD-8654D3E63A97}">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="27.41796875" bestFit="1" customWidth="1"/>
@@ -3238,7 +3266,7 @@
         <v>2</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3260,7 +3288,7 @@
       </c>
       <c r="H8">
         <f>G8*H7</f>
-        <v>6400</v>
+        <v>12800</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3510,6 +3538,11 @@
     <row r="39" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>